<commit_message>
survey_v26: apply second-pass coding corrections (87% omit threshold, 3/46 report all four)
</commit_message>
<xml_diff>
--- a/outputs/survey_v26/Supplementary_data_S2_literature_survey.xlsx
+++ b/outputs/survey_v26/Supplementary_data_S2_literature_survey.xlsx
@@ -428,7 +428,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Supplementary data S2 — literature survey of reporting practice in LIDC-IDRI / LUNA16 lung nodule segmentation</t>
+          <t>Supplementary data — literature survey of reporting practice in LIDC-IDRI / LUNA16 lung nodule segmentation</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Full text: Europe PMC fullTextXML or NCBI PMC (efetch/HTML). Quotations are taken from those renderings; inline mathematics may appear as plain text.</t>
+          <t>Full text: Europe PMC fullTextXML or NCBI PMC rendering. Quotations are taken from those renderings; inline mathematics may appear as plain text.</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  threshold — is the binarisation threshold (value, argmax, level set or selection procedure) stated?</t>
+          <t xml:space="preserve">  threshold — is the binarisation threshold (value, argmax, level set or selection procedure) stated for the final mask?</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rater: single rater; field extraction assisted by a generative AI tool. Each coded field is accompanied by the verbatim supporting passage(s).</t>
+          <t>Rater: single rater. Each coded field is accompanied by the verbatim supporting passage(s).</t>
         </is>
       </c>
     </row>
@@ -3095,11 +3095,7 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Research Square</t>
-        </is>
-      </c>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>A Bayesian TransUNet for Uncertainty-AwareSegmentation of Pulmonary Nodules in CT Scans</t>
@@ -4404,11 +4400,7 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Preprints.org</t>
-        </is>
-      </c>
+      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>DEHA-Net: Dual-Encoder based Hard Attention Network with Adaptive ROI Mechanism for Lung Nodule Segmentation</t>
@@ -4555,11 +4547,7 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>medRxiv</t>
-        </is>
-      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>Early Detection of Lung Cancer in the NLST Dataset*</t>
@@ -5175,11 +5163,7 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Preprints.org</t>
-        </is>
-      </c>
+      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>Multi-center Validation of Pulmonary Nodule Classification Model for Lung Cancer Screening</t>
@@ -6284,11 +6268,7 @@
           <t>2019</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Preprints.org</t>
-        </is>
-      </c>
+      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>Lungs Nodule Detection Using Semantic Segmentation and Classification with Optimal Features</t>
@@ -7222,11 +7202,7 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Research Square</t>
-        </is>
-      </c>
+      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>CNN based pulmonary nodule segmentation using lung-range-standardization</t>
@@ -8441,11 +8417,7 @@
           <t>2020</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>bioRxiv</t>
-        </is>
-      </c>
+      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>An automatic and efficient pulmonary nodule detection system based on multi-model ensemble</t>
@@ -8706,11 +8678,7 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>Research Square</t>
-        </is>
-      </c>
+      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>Segmentation of Pulmonary Nodules Using SegNet and Adversarial Networks</t>
@@ -9290,7 +9258,7 @@
     <col width="9.9" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="36.9" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
     <col width="31.5" customWidth="1" min="14" max="14"/>
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="15.3" customWidth="1" min="16" max="16"/>
@@ -9301,7 +9269,7 @@
     <col width="60" customWidth="1" min="21" max="21"/>
     <col width="60" customWidth="1" min="22" max="22"/>
     <col width="60" customWidth="1" min="23" max="23"/>
-    <col width="58.5" customWidth="1" min="24" max="24"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10610,12 +10578,12 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>stated</t>
+          <t>not stated</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.5 (core map); final SDF thresholded</t>
+          <t>0.5 applies to the intermediate core map only; level of the final SDF threshold not stated</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -10641,7 +10609,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -10660,7 +10628,11 @@
         </is>
       </c>
       <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>second check: final mask from a thresholded SDF whose level is not given</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10756,7 +10728,7 @@
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ; fully automatic: ROI from nnU-Net output</t>
+          <t>fully automatic: ROI from nnU-Net output</t>
         </is>
       </c>
     </row>
@@ -13126,7 +13098,7 @@
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ; initial 2-D ROI supplied (radiologist/GT)</t>
+          <t>initial 2-D ROI supplied (radiologist/GT)</t>
         </is>
       </c>
     </row>

</xml_diff>